<commit_message>
Docs: move the leftover flora details into the regions table
The six details only world-building.md had now sit in the matching
spreadsheet columns, so the doc's flora table keeps just region, flora
and silhouette shape.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nzd-regions.xlsx
+++ b/nzd-regions.xlsx
@@ -745,7 +745,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>Surviving here is unexplained</t>
+          <t>Most basic crawling flora on N-Z-D; surviving here is unexplained</t>
         </is>
       </c>
       <c r="AK2" s="2" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>smaller, simpler version of itself; bendy but robust; symbol of peace and friendship</t>
+          <t>smaller, simpler version of itself; bendy but robust, like banana leaves; symbol of peace and friendship</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="AJ12" s="2" t="inlineStr">
         <is>
-          <t>Slimy, soft; melts ice surfaces with body heat to slide; releases tendrils</t>
+          <t>Slimy, soft; melts ice surfaces with body heat to slide; releases tendrils; one of the few flora that can survive the cold</t>
         </is>
       </c>
       <c r="AK12" s="2" t="inlineStr"/>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>long thin edible strands</t>
+          <t>long thin edible strands, like ultra-slim bananas</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1928,7 +1928,7 @@
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="inlineStr">
         <is>
-          <t>Attaches (to flora or non-flora)</t>
+          <t>Attaches with tendrils through its hole (to flora or non-flora)</t>
         </is>
       </c>
       <c r="AH13" s="2" t="inlineStr"/>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>said to bring good luck</t>
+          <t>only sometimes yielded; said to bring good luck</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2353,7 +2353,7 @@
       <c r="AK17" s="2" t="inlineStr"/>
       <c r="AL17" s="2" t="inlineStr">
         <is>
-          <t>Full of life</t>
+          <t>Full of life; the N-Z-D equivalent of a rainforest</t>
         </is>
       </c>
     </row>

</xml_diff>